<commit_message>
Add accumulated project files: notebooks, docs, tools, data products
Includes new notebooks (011-012b series: bot tracking, numeric testbed,
skew-t experiments), session docs, data products, tool updates, and
reference materials accumulated since last commit.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jupyter/openrouter_cost_history.xlsx
+++ b/jupyter/openrouter_cost_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,37 @@
       </c>
       <c r="I2" t="n">
         <v>37.54539161399998</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-08 09:03:43</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>544.2246</v>
+      </c>
+      <c r="C3" t="n">
+        <v>496.527369536</v>
+      </c>
+      <c r="D3" t="n">
+        <v>47.69723046399997</v>
+      </c>
+      <c r="E3" t="n">
+        <v>170</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2805719439058822</v>
+      </c>
+      <c r="G3" t="n">
+        <v>287</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2970126204808361</v>
+      </c>
+      <c r="I3" t="n">
+        <v>85.24262207799995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>